<commit_message>
feat(web): workspace/market 通知鈴鐺與 notification-service client
- notification-service OpenAPI codegen（swagger-typescript-api）+
  api/index.ts 匯出 notificationApi（OIDC Bearer 注入）
- NotificationBell：未讀數輪詢（60s）、通知下拉、單筆/全部已讀，
  依 type + camelCase payload 配 i18n 渲染
- workspace-web 取代頂欄假鈴鐺；market-web 登入時顯示於導覽列
- i18n 新增 notifications 命名空間（zh-TW / en，xlsx 已同步）

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DNNMi2ZkjM2mZk31yhk25E
</commit_message>
<xml_diff>
--- a/apps/market-web/i18n.xlsx
+++ b/apps/market-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="454">
   <si>
     <t>key</t>
   </si>
@@ -1283,6 +1283,96 @@
   </si>
   <si>
     <t>Got it</t>
+  </si>
+  <si>
+    <t>notifications.title</t>
+  </si>
+  <si>
+    <t>通知</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>notifications.empty</t>
+  </si>
+  <si>
+    <t>目前沒有通知</t>
+  </si>
+  <si>
+    <t>No notifications yet</t>
+  </si>
+  <si>
+    <t>notifications.loading</t>
+  </si>
+  <si>
+    <t>載入中…</t>
+  </si>
+  <si>
+    <t>Loading…</t>
+  </si>
+  <si>
+    <t>notifications.markAllRead</t>
+  </si>
+  <si>
+    <t>全部標為已讀</t>
+  </si>
+  <si>
+    <t>Mark all as read</t>
+  </si>
+  <si>
+    <t>notifications.justNow</t>
+  </si>
+  <si>
+    <t>剛剛</t>
+  </si>
+  <si>
+    <t>Just now</t>
+  </si>
+  <si>
+    <t>notifications.minsAgo</t>
+  </si>
+  <si>
+    <t>{n} 分鐘前</t>
+  </si>
+  <si>
+    <t>{n} min ago</t>
+  </si>
+  <si>
+    <t>notifications.hoursAgo</t>
+  </si>
+  <si>
+    <t>{n} 小時前</t>
+  </si>
+  <si>
+    <t>{n} hr ago</t>
+  </si>
+  <si>
+    <t>notifications.daysAgo</t>
+  </si>
+  <si>
+    <t>{n} 天前</t>
+  </si>
+  <si>
+    <t>{n} days ago</t>
+  </si>
+  <si>
+    <t>notifications.catalogPublished</t>
+  </si>
+  <si>
+    <t>{storeName} 上架了新商品「{catalogName}」</t>
+  </si>
+  <si>
+    <t>{storeName} released a new product "{catalogName}"</t>
+  </si>
+  <si>
+    <t>notifications.storeAnnouncement</t>
+  </si>
+  <si>
+    <t>{storeName}：{title}</t>
+  </si>
+  <si>
+    <t>{storeName}: {title}</t>
   </si>
 </sst>
 </file>
@@ -1668,7 +1758,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C151"/>
+  <dimension ref="A1:C161"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -3336,6 +3426,116 @@
         <v>423</v>
       </c>
     </row>
+    <row r="152" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>